<commit_message>
#8 Simplifica e padroniza o dicionário de dados
</commit_message>
<xml_diff>
--- a/target/avaliacao_01/dicionario_lucimar_oliveira_do_nascimento.xlsx
+++ b/target/avaliacao_01/dicionario_lucimar_oliveira_do_nascimento.xlsx
@@ -7,14 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base consolidada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variáveis analíticas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dicionário de dados" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Base consolidada'!$A$1:$G$26</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Base consolidada'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Variáveis analíticas'!$A$1:$G$21</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Variáveis analíticas'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dicionário de dados'!$A$1:$G$26</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Dicionário de dados'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -175,24 +172,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DicionarioBaseConsolidada" displayName="DicionarioBaseConsolidada" ref="A1:G26" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DicionarioDeDados" displayName="DicionarioDeDados" ref="A1:G26" headerRowCount="1">
   <autoFilter ref="A1:G26"/>
-  <tableColumns count="7">
-    <tableColumn id="1" name="Variável"/>
-    <tableColumn id="2" name="Nome Descritivo"/>
-    <tableColumn id="3" name="Tipo de Dado"/>
-    <tableColumn id="4" name="Unidade de Medida"/>
-    <tableColumn id="5" name="Domínio / Categoria"/>
-    <tableColumn id="6" name="Descrição / Significado"/>
-    <tableColumn id="7" name="Observações"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DicionarioVariaveisAnaliticas" displayName="DicionarioVariaveisAnaliticas" ref="A1:G21" headerRowCount="1">
-  <autoFilter ref="A1:G21"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Variável"/>
     <tableColumn id="2" name="Nome Descritivo"/>
@@ -557,7 +538,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -594,7 +575,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -631,7 +612,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -668,7 +649,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -705,7 +686,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -742,7 +723,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -779,7 +760,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Numérico (inteiro anulável)</t>
+          <t>Numérico (inteiro)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -816,7 +797,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -853,7 +834,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -890,7 +871,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Data/hora após conversão</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -927,7 +908,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Data/hora após conversão</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -964,7 +945,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1001,7 +982,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1038,7 +1019,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Data/hora após conversão</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1075,7 +1056,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Data/hora após conversão</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1112,7 +1093,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1149,7 +1130,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1186,7 +1167,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1223,7 +1204,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1260,7 +1241,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Booleano anulável após conversão</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1297,7 +1278,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Booleano anulável após conversão</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1408,7 +1389,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Categórico (texto)</t>
+          <t>Categórico (nominal)</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1445,7 +1426,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Numérico (inteiro anulável)</t>
+          <t>Numérico (inteiro)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1477,809 +1458,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:G21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="64" customWidth="1" min="6" max="6"/>
-    <col width="72" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Variável</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Nome Descritivo</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Tipo de Dado</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Unidade de Medida</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Domínio / Categoria</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Descrição / Significado</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Observações</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>sg_empresa_icao</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Sigla da Empresa Aérea (ICAO)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Categórico (texto)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Código ICAO; exemplo observado: AAL</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Identificador da companhia no CSV.</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Origem: companhia_icao. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>nr_voo</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Número do Voo</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Categórico (texto)</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Texto; exemplo: 0904</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Identificador comercial do voo.</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Origem: numero_voo. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>sg_icao_origem</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Aeroporto de Origem (ICAO)</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Categórico (texto)</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Código ICAO; exemplo observado: SBGL</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Identificador ICAO do aeródromo de origem.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Origem: origem_icao. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>sg_icao_destino</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Aeroporto de Destino (ICAO)</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Categórico (texto)</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Código ICAO; exemplo observado: SBGL</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Identificador ICAO do aeródromo de destino.</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Origem: destino_icao. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>rota</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Rota / Par Origem-Destino</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Categórico (nominal)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Texto ORIGEM-DESTINO ou ausente</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Par direcional combinando o aeródromo de origem e o de destino</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Derivada de sg_icao_origem + '-' + sg_icao_destino; ausente se qualquer componente faltar. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>dt_partida_prevista</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Data e Horário Previsto de Partida</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Data/hora após conversão</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>AAAA-MM-DD HH:MM:SS ou ausente</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Timestamp registrado de partida prevista.</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Origem: partida_prevista. Fuso não informado no CSV. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>dt_partida_real</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Data e Horário Real de Partida</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Data/hora após conversão</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>AAAA-MM-DD HH:MM:SS ou ausente</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Timestamp registrado de partida real.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Origem: partida_real. Fuso não informado no CSV. Informação de desfecho; excluir de X na previsão pré-voo. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>dt_chegada_prevista</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Data e Horário Previsto de Chegada</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Data/hora após conversão</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>AAAA-MM-DD HH:MM:SS ou ausente</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Timestamp registrado de chegada prevista.</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Origem: chegada_prevista. Fuso não informado no CSV. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>dt_chegada_real</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Data e Horário Real de Chegada</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Data/hora após conversão</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>AAAA-MM-DD HH:MM:SS ou ausente</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Timestamp registrado de chegada real.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Origem: chegada_real. Fuso não informado no CSV. Informação de desfecho; excluir de X na previsão pré-voo. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Ano da Operação</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Numérico (inteiro)</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Ano</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Ano civil; validar cobertura na base completa</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Ano da Operação extraído(a) do timestamp previsto de partida.</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Derivada de dt_partida_prevista; ausente se data inválida ou ausente. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>mes</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Mês da Operação</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Numérico (inteiro)</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Mês</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>1 a 12</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Mês da Operação extraído(a) do timestamp previsto de partida.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Derivada de dt_partida_prevista; ausente se data inválida ou ausente. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>dia_semana</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Dia da Semana da Partida</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Categórico (ordinal)</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>0 a 6 (0=Segunda ... 6=Domingo)</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Dia da Semana da Partida extraído(a) do timestamp previsto de partida.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Derivada de dt_partida_prevista; ausente se data inválida ou ausente. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>hora_partida_prevista</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Hora Programada de Partida</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Numérico (inteiro)</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Horas</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>0 a 23</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Hora Programada de Partida extraído(a) do timestamp previsto de partida.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Derivada de dt_partida_prevista; ausente se data inválida ou ausente. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>minuto_partida_previsto</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Minuto Programado de Partida</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Numérico (inteiro)</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Minutos</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>0 a 59</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Minuto Programado de Partida extraído(a) do timestamp previsto de partida.</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Derivada de dt_partida_prevista; ausente se data inválida ou ausente. Candidata pré-voo: validar disponibilidade e versão histórica no instante da previsão. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>tempo_voo_planejado_minutos</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Diferença bruta entre horários previstos</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Numérico (contínuo)</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Minutos</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Real com sinal ou ausente; sem faixa validada</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>(dt_chegada_prevista - dt_partida_prevista).total_seconds() / 60; diferença bruta entre timestamps.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Fusos e comparabilidade temporal não comprovados, sobretudo em voos internacionais. Não interpretar como duração efetiva; excluir de X até validação. Preservar ausentes e investigar valores negativos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>cd_situacao_voo</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Situação Operacional do Voo</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Categórico (texto)</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Observados: REALIZADO, CANCELADO</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Situação operacional registrada no CSV.</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Origem: situacao_voo. Informação de desfecho; excluir de X na previsão pré-voo. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>atraso_partida_minutos</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Tempo Líquido de Atraso na Partida</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Numérico (contínuo)</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Minutos</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Real com sinal ou ausente; sem corte automático</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>(dt_partida_real - dt_partida_prevista).total_seconds() / 60.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Derivada para auditoria e construção dos alvos; comparar com atraso_partida_min. Investigar extremos e datas inconsistentes. Informação de desfecho; excluir de X na previsão pré-voo. Preservar ausentes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="75" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>faixa_atraso_partida</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Faixa Ordinal de Atraso na Partida (Target Principal)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Categórico (ordinal)</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>0: Pontual ou antecipado (x≤0); 1: Atraso inferior a 15 min (0&lt;x&lt;15); 2: Atraso de 15 a 30 min (15≤x≤30); 3: Atraso superior a 30 até 45 min (30&lt;x≤45); 4: Atraso superior a 45 até 60 min (45&lt;x≤60); 5: Atraso superior a 60 min (x&gt;60).</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Alvo principal ordinal de seis classes, definido pelo estudo sobre atraso_partida_minutos (x).</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Rótulo textual ordenado; código numérico em codigo_faixa_atraso. Sem classificação para não realizados ou atraso indisponível. Não usar em X; limiares operacionais do estudo, sem atribuição normativa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>atraso_bi</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Indicador de Atraso Binário (Target Secundário)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Inteiro anulável (alvo binário)</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>0, 1 ou ausente</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Alvo secundário: 1 se atraso_partida_minutos ≥15; 0 se &lt;15, entre realizados com atraso disponível.</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Limiar definido neste estudo. Ausente para não realizados ou atraso indisponível; não substituir ausentes por 0. Excluir de X.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>codigo_faixa_atraso</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Código ordinal da faixa de atraso</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Inteiro anulável (ordinal)</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Não aplicável</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>0, 1, 2, 3, 4, 5 ou ausente</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Codificação de faixa_atraso_partida, preservando exatamente os seis intervalos definidos na linha do alvo principal.</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Alvo numérico principal; ausente para não realizados ou atraso indisponível. Excluir de X.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G21"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>